<commit_message>
Adiciona aba de preços na planilha (Ondansetrona 8mg)
</commit_message>
<xml_diff>
--- a/data/produtos_up_totalfarma.xlsx
+++ b/data/produtos_up_totalfarma.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet name="Produtos UP Total Farma" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resumo por Categoria" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Preços" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produtos UP Total Farma'!$A$1:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +44,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +61,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F7F4"/>
         <bgColor rgb="00F2F7F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBF3F7"/>
+        <bgColor rgb="00FBF3F7"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -103,6 +111,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1553,4 +1564,159 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID Produto</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Apresentação</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Menor Preço (R$)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Maior Preço (R$)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Onde achou menor</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Onde achou maior</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Fontes da pesquisa</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Data da pesquisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Ondansetrona 8 mg orodispersível</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>10 comprimidos orodispersíveis</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>14.28</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Consulta Remédios (agregador)</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Pague Menos (gen. Pharlab)</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Droga Raia, Drogasil, Pague Menos, Consulta Remédios, Panvel, Ultrafarma</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Ondansetrona 8 mg orodispersível</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>30 comprimidos orodispersíveis</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>33.63</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>141.13</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Ultrafarma (gen. Prati-Donaduzzi, Pix)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Drogaria São João (gen. Althaia)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Ultrafarma, Preço Popular, Drogaria São Paulo, Drogaria São João, Panvel</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona precos.json (fonte) + planilha com Ondansetrona 4mg
</commit_message>
<xml_diff>
--- a/data/produtos_up_totalfarma.xlsx
+++ b/data/produtos_up_totalfarma.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produtos UP Total Farma'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -106,9 +106,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1404,7 +1401,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Indicado p/ febre e dores leves; contraindicado com ácido acetilsalicílico ou AINE (história de alergia, úlcera, últimos 3 meses de gravidez)</t>
+          <t>Indicado p/ febre e dores leves; contraindicado com ácido acetilsalicílico ou AINE</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1429,7 +1426,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Provável à base de ácido acetilsalicílico ou dipirona/AINE. Não indicado p/ menores de 12 anos. Barcode 7891142982407.</t>
+          <t>Não indicado p/ menores de 12 anos. Barcode 7891142982407.</t>
         </is>
       </c>
     </row>
@@ -1500,12 +1497,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Quantidade</t>
         </is>
@@ -1552,12 +1549,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1572,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1634,41 +1631,41 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Ondansetrona 8 mg orodispersível</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>10 comprimidos orodispersíveis</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n">
+      <c r="D2" s="5" t="n">
         <v>14.28</v>
       </c>
-      <c r="E2" s="6" t="n">
+      <c r="E2" s="5" t="n">
         <v>51.12</v>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Consulta Remédios (agregador)</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Pague Menos (gen. Pharlab)</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Droga Raia, Drogasil, Pague Menos, Consulta Remédios, Panvel, Ultrafarma</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
@@ -1715,8 +1712,90 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Ondansetrona 4 mg orodispersível</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>10 comprimidos orodispersíveis</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>14.28</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Consulta Remédios (agregador)</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia (gen. Neo Química)</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia, Drogasil, Pague Menos, Farma Conde, Ultrafarma, Consulta Remédios</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Ondansetrona 4 mg orodispersível</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>30 comprimidos orodispersíveis</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>47.83</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>77.34</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Consulta Remédios (agregador)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Pague Menos (gen. Biolab)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Droga Raia, Drogasil, Pague Menos, Ultrafarma, Consulta Remédios</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
+  <autoFilter ref="A1:I5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona Embeleze Natu Cor no precos.json + planilha
</commit_message>
<xml_diff>
--- a/data/produtos_up_totalfarma.xlsx
+++ b/data/produtos_up_totalfarma.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produtos UP Total Farma'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1569,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1794,8 +1794,49 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Embeleze Natu Cor (tintura vegana sem amônia)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>1 unidade (tom variável, ex.: 1.0 Preto Natural)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>20.88</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Drogaria Venâncio (tom 1.0, 20% off)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Magazine Luiza (tom 5.0, Pix)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Embelleze (site), Mercado Livre, Drogaria Venâncio, Drogaria São Paulo, Drogarias Minas Mais, Araujo, Drogarias Pacheco, Magazine Luiza, Drogasil</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I5"/>
+  <autoFilter ref="A1:I6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Consolida ondansetrona 4/8mg em 1 produto + checagem anti-duplicidade
</commit_message>
<xml_diff>
--- a/data/produtos_up_totalfarma.xlsx
+++ b/data/produtos_up_totalfarma.xlsx
@@ -1636,19 +1636,19 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Ondansetrona 8 mg orodispersível</t>
+          <t>Ondansetrona orodispersível</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>10 comprimidos orodispersíveis</t>
+          <t>4 mg - 10 comprimidos orodispersíveis</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
         <v>14.28</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>51.12</v>
+        <v>25.6</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -1657,12 +1657,12 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Pague Menos (gen. Pharlab)</t>
+          <t>Droga Raia (gen. Neo Química)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Droga Raia, Drogasil, Pague Menos, Consulta Remédios, Panvel, Ultrafarma</t>
+          <t>Droga Raia, Drogasil, Pague Menos, Farma Conde, Ultrafarma, Consulta Remédios</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -1677,33 +1677,33 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Ondansetrona 8 mg orodispersível</t>
+          <t>Ondansetrona orodispersível</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>30 comprimidos orodispersíveis</t>
+          <t>4 mg - 30 comprimidos orodispersíveis</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>33.63</v>
+        <v>47.83</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>141.13</v>
+        <v>77.34</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Ultrafarma (gen. Prati-Donaduzzi, Pix)</t>
+          <t>Consulta Remédios (agregador)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Drogaria São João (gen. Althaia)</t>
+          <t>Pague Menos (gen. Biolab)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Ultrafarma, Preço Popular, Drogaria São Paulo, Drogaria São João, Panvel</t>
+          <t>Droga Raia, Drogasil, Pague Menos, Ultrafarma, Consulta Remédios</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -1714,23 +1714,23 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Ondansetrona 4 mg orodispersível</t>
+          <t>Ondansetrona orodispersível</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>10 comprimidos orodispersíveis</t>
+          <t>8 mg - 10 comprimidos orodispersíveis</t>
         </is>
       </c>
       <c r="D4" s="5" t="n">
         <v>14.28</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25.6</v>
+        <v>51.12</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Droga Raia (gen. Neo Química)</t>
+          <t>Pague Menos (gen. Pharlab)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Droga Raia, Drogasil, Pague Menos, Farma Conde, Ultrafarma, Consulta Remédios</t>
+          <t>Droga Raia, Drogasil, Pague Menos, Consulta Remédios, Panvel, Ultrafarma</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -1755,37 +1755,37 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Ondansetrona 4 mg orodispersível</t>
+          <t>Ondansetrona orodispersível</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>30 comprimidos orodispersíveis</t>
+          <t>8 mg - 30 comprimidos orodispersíveis</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>47.83</v>
+        <v>33.63</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>77.34</v>
+        <v>141.13</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Consulta Remédios (agregador)</t>
+          <t>Ultrafarma (gen. Prati-Donaduzzi, Pix)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Pague Menos (gen. Biolab)</t>
+          <t>Drogaria São João (gen. Althaia)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Droga Raia, Drogasil, Pague Menos, Ultrafarma, Consulta Remédios</t>
+          <t>Ultrafarma, Preço Popular, Drogaria São Paulo, Drogaria São João, Panvel</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -1796,7 +1796,7 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Adiciona L'Oréal Casting Creme Gloss no precos.json + planilha
</commit_message>
<xml_diff>
--- a/data/produtos_up_totalfarma.xlsx
+++ b/data/produtos_up_totalfarma.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produtos UP Total Farma'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1569,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1835,8 +1835,49 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>L'Oréal Paris Casting Creme Gloss (tintura sem amônia)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>1 unidade (tom variável, ex.: 600 Louro Escuro)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>20.07</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>58.55</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Drogaria São Paulo (tom 400 Castanho Natural)</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Magazine Luiza (tom 600, tonalizante)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Amazon, L'Oréal (site), Drogarias Pacheco, Ultrafarma, Magazine Luiza, Droga Raia, Drogasil, Drogaria São Paulo, Farmácia Indiana, Pague Menos, Drogaria Shopper</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
+  <autoFilter ref="A1:I7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona Wella Koleston Deluxe no precos.json + planilha
</commit_message>
<xml_diff>
--- a/data/produtos_up_totalfarma.xlsx
+++ b/data/produtos_up_totalfarma.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produtos UP Total Farma'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1569,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1876,8 +1876,49 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Wella Koleston Deluxe (tintura permanente 0% amônia)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>1 unidade (tom variável, ex.: 60 Louro Escuro)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Promoção de farmácia (Instagram, R$ 24,99)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Shopee (variações R$ 51,90-55,90)</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Loja Wella, Mercado Livre, Shopee, Lojas Rede, Magazine Luiza, Buscapé, Pacheco, Drogaria São Paulo, Stylosa, Farmagerty, Instagram promo</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I7"/>
+  <autoFilter ref="A1:I8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona Cor & Ton Mega Colors no precos.json + planilha
</commit_message>
<xml_diff>
--- a/data/produtos_up_totalfarma.xlsx
+++ b/data/produtos_up_totalfarma.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produtos UP Total Farma'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1569,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1917,8 +1917,49 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Cor &amp; Ton Mega Colors (Niely - tintura permanente)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>1 unidade (tom variável, ex.: 6.646 Vermelho Cereja)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>34.99</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Nossa Farma (tom 12.111 Louro Super Platinado)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Drogarias Pacheco (tom 12.111)</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Drogaria São Paulo, Farmácias Nogueira, Mega Farma, Farmanello, Nossa Farma, Drogaria Retiro, Descontão, Cliquefarma, Goya Perfumaria, Amazon, Lumina Web, Pacheco, Goiás Atacado</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I8"/>
+  <autoFilter ref="A1:I9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Completa pesquisa de preços (14 produtos)
</commit_message>
<xml_diff>
--- a/data/produtos_up_totalfarma.xlsx
+++ b/data/produtos_up_totalfarma.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produtos UP Total Farma'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Preços'!$A$1:$I$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1569,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1958,8 +1958,373 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>L'Oréal Paris Nutrisse (tintura permanente)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>1 unidade (tom variável, ex.: 81 Louro Paixão Nacional)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Promoção L'Oréal Paris (Instagram, R$ 26,90)</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Mercado Livre (Nutrisse permanente)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia, Mercado Livre, Droga Cristal 24h, Goyaperfumaria, L'Oréal Paris (site), Instagram promo</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Wella Koleston (linha padrão, tintura permanente)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>1 unidade (tom variável, ex.: 20 Preto)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>22.95</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>36.48</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Promoção de farmácia (Instagram, De R$ 25,95 por R$ 22,95)</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Droga Raia (loja parceira, tom 20 Preto)</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Droga Raia, Drogasil, Pacheco, Instagram promo, Wella (site), Farmácia Permanente</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>L'Oréal Paris Excellence Creme (Imédia Excellence)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>1 unidade (tom variável, ex.: 1 Preto / 7.1 Louro Acinzentado)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>25.09</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>53.53</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Drogasil (via Melhora o Preço, R$ 25,09)</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia (tom 7.1 Louro Acinzentado)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia, Drogasil, Mercado Livre, eBay, Melhora o Preço, L'Oréal Paris (site/PT)</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Garnier Nutrisse (tintura permanente)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>1 unidade (tom variável, ex.: 100 Louro Sol / 50 Amêndoa)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>26.99</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Ultrafarma / Shopper (R$ 26,99)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Drogaria São João (R$ 29,99)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Droga Raia, Drogasil, Drogaria São João, Ultrafarma, Shopper, Magazine Luiza, Garnier (site)</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Expec Xarope Tripla Ação 120 mL</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Xarope 120 mL</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>56.58</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Drogasil (R$ 27,90)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Drogarias Pacheco (R$ 56,58)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia, Drogasil, Drogaria São Paulo, Pacheco, Pague Menos, Ultrafarma</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Lavitan (linha de vitaminas/suplementos)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>1 unidade (variável por tipo: Vit D, A-Z, etc.)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>39.59</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Drogaria São João (Vitamina D Cimed, R$ 19,99)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Drogaria São Paulo (Lavitan 0,21mg, R$ 39,59)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Droga Raia, Drogasil, Drogaria São Paulo, Drogaria São João, Panvel, lavitan.com.br</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Ibuprofeno 400 mg (Alivium) - cápsulas</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>10 cápsulas (400 mg)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>26.99</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>33.48</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia / Farmácia Modelo (R$ 26,99)</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Qualidoc (R$ 33,48)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia, Ultrafarma, Farmácia Modelo, Preço Popular, Drogaria Venâncio, Qualidoc</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Cápsula 'ESFENO...' (marca a confirmar)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Não localizado</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Não localizado</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Busca por barcode 78963317034311 (sem resultado)</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Ibuprofeno Suspensão Gotas 100 mg/mL</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Suspensão gotas 20 mL (100 mg/mL)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Droga Raia (Nova Química, R$ 6,99)</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Drogaria Venâncio (Geolab, R$ 8,49)</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Drogasil, Droga Raia, Drogaria São Paulo, Drogaria Venâncio, Pague Menos, Consulta Remédios</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I9"/>
+  <autoFilter ref="A1:I18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>